<commit_message>
chore: regenerate mock rosters with single DOB column
</commit_message>
<xml_diff>
--- a/mockdata/import-samples/roster-ป.1-1.xlsx
+++ b/mockdata/import-samples/roster-ป.1-1.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:E14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,15 +410,9 @@
         <v>นามสกุล</v>
       </c>
       <c r="D1" t="str">
-        <v>วันเกิด-วัน</v>
+        <v>วันเกิด</v>
       </c>
       <c r="E1" t="str">
-        <v>วันเกิด-เดือน</v>
-      </c>
-      <c r="F1" t="str">
-        <v>วันเกิด-ปี(พ.ศ.)</v>
-      </c>
-      <c r="G1" t="str">
         <v>เพศ</v>
       </c>
     </row>
@@ -432,16 +426,10 @@
       <c r="C2" t="str">
         <v>ชัยชนะ</v>
       </c>
-      <c r="D2">
-        <v>11</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>2563</v>
-      </c>
-      <c r="G2" t="str">
+      <c r="D2" t="str">
+        <v>11/4/2563</v>
+      </c>
+      <c r="E2" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -455,16 +443,10 @@
       <c r="C3" t="str">
         <v>ศักดิ์ดี</v>
       </c>
-      <c r="D3">
-        <v>21</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>2563</v>
-      </c>
-      <c r="G3" t="str">
+      <c r="D3" t="str">
+        <v>21/4/2563</v>
+      </c>
+      <c r="E3" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -478,16 +460,10 @@
       <c r="C4" t="str">
         <v>ชัยชนะ</v>
       </c>
-      <c r="D4">
-        <v>25</v>
-      </c>
-      <c r="E4">
-        <v>8</v>
-      </c>
-      <c r="F4">
-        <v>2563</v>
-      </c>
-      <c r="G4" t="str">
+      <c r="D4" t="str">
+        <v>25/8/2563</v>
+      </c>
+      <c r="E4" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -501,16 +477,10 @@
       <c r="C5" t="str">
         <v>หอมดี</v>
       </c>
-      <c r="D5">
-        <v>22</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>2563</v>
-      </c>
-      <c r="G5" t="str">
+      <c r="D5" t="str">
+        <v>22/4/2563</v>
+      </c>
+      <c r="E5" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -524,16 +494,10 @@
       <c r="C6" t="str">
         <v>แสงดาว</v>
       </c>
-      <c r="D6">
-        <v>18</v>
-      </c>
-      <c r="E6">
-        <v>7</v>
-      </c>
-      <c r="F6">
-        <v>2563</v>
-      </c>
-      <c r="G6" t="str">
+      <c r="D6" t="str">
+        <v>18/7/2563</v>
+      </c>
+      <c r="E6" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -547,16 +511,10 @@
       <c r="C7" t="str">
         <v>ยิ้มแย้ม</v>
       </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>2563</v>
-      </c>
-      <c r="G7" t="str">
+      <c r="D7" t="str">
+        <v>10/5/2563</v>
+      </c>
+      <c r="E7" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -570,16 +528,10 @@
       <c r="C8" t="str">
         <v>หอมดี</v>
       </c>
-      <c r="D8">
-        <v>21</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>2563</v>
-      </c>
-      <c r="G8" t="str">
+      <c r="D8" t="str">
+        <v>21/1/2563</v>
+      </c>
+      <c r="E8" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -593,16 +545,10 @@
       <c r="C9" t="str">
         <v>ศักดิ์ดี</v>
       </c>
-      <c r="D9">
-        <v>12</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>2563</v>
-      </c>
-      <c r="G9" t="str">
+      <c r="D9" t="str">
+        <v>12/1/2563</v>
+      </c>
+      <c r="E9" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -616,16 +562,10 @@
       <c r="C10" t="str">
         <v>รักดี</v>
       </c>
-      <c r="D10">
-        <v>26</v>
-      </c>
-      <c r="E10">
-        <v>4</v>
-      </c>
-      <c r="F10">
-        <v>2563</v>
-      </c>
-      <c r="G10" t="str">
+      <c r="D10" t="str">
+        <v>26/4/2563</v>
+      </c>
+      <c r="E10" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -639,16 +579,10 @@
       <c r="C11" t="str">
         <v>ดีงาม</v>
       </c>
-      <c r="D11">
-        <v>8</v>
-      </c>
-      <c r="E11">
-        <v>5</v>
-      </c>
-      <c r="F11">
-        <v>2563</v>
-      </c>
-      <c r="G11" t="str">
+      <c r="D11" t="str">
+        <v>8/5/2563</v>
+      </c>
+      <c r="E11" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -662,16 +596,10 @@
       <c r="C12" t="str">
         <v>สุขใส</v>
       </c>
-      <c r="D12">
-        <v>17</v>
-      </c>
-      <c r="E12">
-        <v>11</v>
-      </c>
-      <c r="F12">
-        <v>2563</v>
-      </c>
-      <c r="G12" t="str">
+      <c r="D12" t="str">
+        <v>17/11/2563</v>
+      </c>
+      <c r="E12" t="str">
         <v>ชาย</v>
       </c>
     </row>
@@ -685,16 +613,10 @@
       <c r="C13" t="str">
         <v>รุ่งเรือง</v>
       </c>
-      <c r="D13">
-        <v>17</v>
-      </c>
-      <c r="E13">
-        <v>7</v>
-      </c>
-      <c r="F13">
-        <v>2563</v>
-      </c>
-      <c r="G13" t="str">
+      <c r="D13" t="str">
+        <v>17/7/2563</v>
+      </c>
+      <c r="E13" t="str">
         <v>หญิง</v>
       </c>
     </row>
@@ -708,22 +630,16 @@
       <c r="C14" t="str">
         <v>ยิ้มแย้ม</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <v>12</v>
-      </c>
-      <c r="F14">
-        <v>2563</v>
-      </c>
-      <c r="G14" t="str">
+      <c r="D14" t="str">
+        <v>1/12/2563</v>
+      </c>
+      <c r="E14" t="str">
         <v>ชาย</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>